<commit_message>
Rewrite case 3 smoke test: unify tab steps via TABS_PLAN loop
- Remove duplicated OCR wait logic, reuse assert_document_created
- Replace 9 copies of _do_tab_step with data-driven loop over TABS_PLAN
- Guard take_screenshot in except block
- Update test case xlsx
</commit_message>
<xml_diff>
--- a/products/Editors/scenarios/smoke/3. Создание нового документа и проверка вкладок на панели инструментов.xlsx
+++ b/products/Editors/scenarios/smoke/3. Создание нового документа и проверка вкладок на панели инструментов.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Testing\Editors\test_cases\smoke\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Testing\products\Editors\scenarios\smoke\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BDB67B9-27FC-4219-A4B4-6E9732092E82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5411607C-7D21-471C-B54A-B52D8D4B2BBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="37">
   <si>
     <t>Расположение</t>
   </si>
@@ -157,6 +157,12 @@
   </si>
   <si>
     <t>Редактор остается запущенным с созданным документом. Вкладка “Плагины” активна</t>
+  </si>
+  <si>
+    <t>Severity</t>
+  </si>
+  <si>
+    <t>HIGH</t>
   </si>
 </sst>
 </file>
@@ -203,7 +209,19 @@
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -217,9 +235,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:G15" totalsRowShown="0">
-  <autoFilter ref="A1:G15" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:H15" totalsRowShown="0">
+  <autoFilter ref="A1:H15" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="8">
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Расположение"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Наименование"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Предусловия"/>
@@ -227,6 +245,7 @@
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Постусловия"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Ожидаемый результат"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Тег"/>
+    <tableColumn id="1" xr3:uid="{082E9623-558E-45E1-84A5-6503D3FE79D2}" name="Severity" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -517,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="50.6640625" style="2" customWidth="1"/>
@@ -530,7 +549,7 @@
     <col min="9" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -552,8 +571,11 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H1" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -577,7 +599,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
@@ -599,8 +621,11 @@
       <c r="G3" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H3" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
@@ -622,8 +647,11 @@
       <c r="G4" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="H4" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -645,8 +673,11 @@
       <c r="G5" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H5" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -668,8 +699,11 @@
       <c r="G6" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H6" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>8</v>
       </c>
@@ -691,8 +725,11 @@
       <c r="G7" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H7" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
@@ -714,8 +751,11 @@
       <c r="G8" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H8" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
@@ -737,8 +777,11 @@
       <c r="G9" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H9" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -760,8 +803,11 @@
       <c r="G10" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H10" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
@@ -783,8 +829,11 @@
       <c r="G11" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H11" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
@@ -806,8 +855,11 @@
       <c r="G12" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H12" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>8</v>
       </c>
@@ -829,8 +881,11 @@
       <c r="G13" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H13" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>8</v>
       </c>
@@ -852,8 +907,11 @@
       <c r="G14" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H14" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="E15" s="1" t="s">
         <v>34</v>
       </c>

</xml_diff>

<commit_message>
Update case 3 xlsx source
</commit_message>
<xml_diff>
--- a/products/Editors/scenarios/smoke/3. Создание нового документа и проверка вкладок на панели инструментов.xlsx
+++ b/products/Editors/scenarios/smoke/3. Создание нового документа и проверка вкладок на панели инструментов.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Testing\products\Editors\scenarios\smoke\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5411607C-7D21-471C-B54A-B52D8D4B2BBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{641C55CB-295F-4F2C-981A-5DDC04B3B933}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,12 +72,6 @@
     <t>Редактор запущен.</t>
   </si>
   <si>
-    <t>Отображается вкладка меню “Главная”.</t>
-  </si>
-  <si>
-    <t>Кликнуть на кнопку “Документ”.</t>
-  </si>
-  <si>
     <t>Панель инструментов.
 Кликнуть по вкладке “Файл”.</t>
   </si>
@@ -163,6 +157,12 @@
   </si>
   <si>
     <t>HIGH</t>
+  </si>
+  <si>
+    <t>Отображается главное окно редактора вкладка меню “Главная”.</t>
+  </si>
+  <si>
+    <t>Кликнуть на “Документ”.</t>
   </si>
 </sst>
 </file>
@@ -572,7 +572,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -642,7 +642,7 @@
         <v>8</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>8</v>
@@ -662,19 +662,19 @@
         <v>8</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -688,19 +688,19 @@
         <v>8</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -714,19 +714,19 @@
         <v>8</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -740,19 +740,19 @@
         <v>8</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -766,19 +766,19 @@
         <v>8</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -792,19 +792,19 @@
         <v>8</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -818,19 +818,19 @@
         <v>8</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -844,19 +844,19 @@
         <v>8</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -870,19 +870,19 @@
         <v>8</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -896,24 +896,24 @@
         <v>8</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="E15" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>